<commit_message>
Refactor README files for clarity and consistency across weeks
</commit_message>
<xml_diff>
--- a/week_2/Input Data.xlsx
+++ b/week_2/Input Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13280" windowHeight="5040" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13280" windowHeight="5040" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="6" r:id="rId1"/>
@@ -269,8 +269,8 @@
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="\₦#,##0"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="\₦#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -482,9 +482,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -497,12 +497,12 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -2165,7 +2165,7 @@
         <v>44066.666666666664</v>
       </c>
       <c r="J11" s="14">
-        <f>D11-E11</f>
+        <f t="shared" ref="J11:J17" si="3">D11-E11</f>
         <v>73333.333333333343</v>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
         <v>41066.666666666664</v>
       </c>
       <c r="J12" s="14">
-        <f>D12-E12</f>
+        <f t="shared" si="3"/>
         <v>36666.666666666679</v>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
         <v>41066.666666666664</v>
       </c>
       <c r="J13" s="14">
-        <f>D13-E13</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
         <v>51533.333333333336</v>
       </c>
       <c r="J14" s="14">
-        <f>D14-E14</f>
+        <f t="shared" si="3"/>
         <v>86666.666666666657</v>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
         <v>48533.333333333336</v>
       </c>
       <c r="J15" s="14">
-        <f>D15-E15</f>
+        <f t="shared" si="3"/>
         <v>43333.333333333321</v>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
         <v>48533.333333333336</v>
       </c>
       <c r="J16" s="14">
-        <f>D16-E16</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2393,7 +2393,7 @@
         <v>36000</v>
       </c>
       <c r="J17" s="25">
-        <f>D17-E17</f>
+        <f t="shared" si="3"/>
         <v>125000</v>
       </c>
     </row>
@@ -2450,26 +2450,26 @@
         <v>100000</v>
       </c>
       <c r="E19" s="23">
-        <f t="shared" ref="E19:E22" si="3">E18</f>
+        <f t="shared" ref="E19:E22" si="4">E18</f>
         <v>25000</v>
       </c>
       <c r="F19" s="24">
-        <f t="shared" ref="F19:F22" si="4">F18</f>
+        <f t="shared" ref="F19:F22" si="5">F18</f>
         <v>6000</v>
       </c>
       <c r="G19" s="24">
         <v>0</v>
       </c>
       <c r="H19" s="25">
-        <f t="shared" ref="H19:H22" si="5">H18</f>
+        <f t="shared" ref="H19:H22" si="6">H18</f>
         <v>25000</v>
       </c>
       <c r="I19" s="25">
-        <f t="shared" ref="I19:I26" si="6">E19+F19</f>
+        <f t="shared" ref="I19:I25" si="7">E19+F19</f>
         <v>31000</v>
       </c>
       <c r="J19" s="25">
-        <f t="shared" ref="J19:J26" si="7">D19-H19</f>
+        <f t="shared" ref="J19:J25" si="8">D19-H19</f>
         <v>75000</v>
       </c>
     </row>
@@ -2484,30 +2484,30 @@
         <v>45970</v>
       </c>
       <c r="D20" s="22">
-        <f t="shared" ref="D20:D23" si="8">D19-H19</f>
+        <f t="shared" ref="D20:D22" si="9">D19-H19</f>
         <v>75000</v>
       </c>
       <c r="E20" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>25000</v>
       </c>
       <c r="F20" s="24">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>6000</v>
       </c>
       <c r="G20" s="24">
         <v>0</v>
       </c>
       <c r="H20" s="25">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>25000</v>
       </c>
       <c r="I20" s="25">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>31000</v>
       </c>
       <c r="J20" s="25">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>50000</v>
       </c>
       <c r="K20" s="14">
@@ -2526,30 +2526,30 @@
         <v>46000</v>
       </c>
       <c r="D21" s="22">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>50000</v>
       </c>
       <c r="E21" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>25000</v>
       </c>
       <c r="F21" s="24">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>6000</v>
       </c>
       <c r="G21" s="24">
         <v>0</v>
       </c>
       <c r="H21" s="25">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>25000</v>
       </c>
       <c r="I21" s="25">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>31000</v>
       </c>
       <c r="J21" s="25">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>25000</v>
       </c>
     </row>
@@ -2564,30 +2564,30 @@
         <v>46031</v>
       </c>
       <c r="D22" s="22">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>25000</v>
       </c>
       <c r="E22" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>25000</v>
       </c>
       <c r="F22" s="24">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>6000</v>
       </c>
       <c r="G22" s="24">
         <v>0</v>
       </c>
       <c r="H22" s="25">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>25000</v>
       </c>
       <c r="I22" s="25">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>31000</v>
       </c>
       <c r="J22" s="25">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
         <v>65966.666666666657</v>
       </c>
       <c r="J23" s="30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>113333.33333333334</v>
       </c>
     </row>
@@ -2660,11 +2660,11 @@
         <v>56666.666666666664</v>
       </c>
       <c r="I24" s="30">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>63466.666666666664</v>
       </c>
       <c r="J24" s="30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>56666.666666666679</v>
       </c>
     </row>
@@ -2698,11 +2698,11 @@
         <v>56666.666666666664</v>
       </c>
       <c r="I25" s="30">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>63466.666666666664</v>
       </c>
       <c r="J25" s="30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2829,6 +2829,34 @@
       <c r="C29" s="18">
         <v>45881</v>
       </c>
+      <c r="D29" s="9">
+        <f>Sheet1!C10</f>
+        <v>80000</v>
+      </c>
+      <c r="E29" s="7">
+        <f>Sheet1!C10/Sheet1!G10</f>
+        <v>26666.666666666668</v>
+      </c>
+      <c r="F29">
+        <f>Sheet1!C10*Sheet1!I10</f>
+        <v>3200</v>
+      </c>
+      <c r="G29">
+        <f>Sheet1!E9</f>
+        <v>1000</v>
+      </c>
+      <c r="H29" s="14">
+        <f>E29+F29</f>
+        <v>29866.666666666668</v>
+      </c>
+      <c r="I29" s="14">
+        <f>E29+F29+G29</f>
+        <v>30866.666666666668</v>
+      </c>
+      <c r="J29" s="14">
+        <f>D29-H29</f>
+        <v>50133.333333333328</v>
+      </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="1" t="s">
@@ -2840,6 +2868,33 @@
       <c r="C30" s="18">
         <v>45912</v>
       </c>
+      <c r="D30" s="9">
+        <f>J29</f>
+        <v>50133.333333333328</v>
+      </c>
+      <c r="E30" s="7">
+        <f>E29</f>
+        <v>26666.666666666668</v>
+      </c>
+      <c r="F30">
+        <f>F29</f>
+        <v>3200</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14">
+        <f>H29</f>
+        <v>29866.666666666668</v>
+      </c>
+      <c r="I30" s="14">
+        <f>E30+F30</f>
+        <v>29866.666666666668</v>
+      </c>
+      <c r="J30" s="14">
+        <f t="shared" ref="J30:J34" si="10">D30-H30</f>
+        <v>20266.666666666661</v>
+      </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="1" t="s">
@@ -2851,6 +2906,33 @@
       <c r="C31" s="18">
         <v>45942</v>
       </c>
+      <c r="D31" s="9">
+        <f>D30-E30</f>
+        <v>23466.666666666661</v>
+      </c>
+      <c r="E31" s="7">
+        <f>E30</f>
+        <v>26666.666666666668</v>
+      </c>
+      <c r="F31">
+        <f>F30</f>
+        <v>3200</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <f>H30</f>
+        <v>29866.666666666668</v>
+      </c>
+      <c r="I31" s="14">
+        <f>E31+F31</f>
+        <v>29866.666666666668</v>
+      </c>
+      <c r="J31" s="14">
+        <f t="shared" si="10"/>
+        <v>-6400.0000000000073</v>
+      </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="1" t="s">
@@ -2862,8 +2944,36 @@
       <c r="C32" s="18">
         <v>45882</v>
       </c>
-    </row>
-    <row r="33" spans="1:3">
+      <c r="D32" s="9">
+        <f>Sheet1!C11</f>
+        <v>100000</v>
+      </c>
+      <c r="E32" s="7">
+        <f>Sheet1!C11/Sheet1!G11</f>
+        <v>33333.333333333336</v>
+      </c>
+      <c r="F32">
+        <f>Sheet1!C11*Sheet1!I11</f>
+        <v>4000</v>
+      </c>
+      <c r="G32">
+        <f>Sheet1!E11</f>
+        <v>3000</v>
+      </c>
+      <c r="H32" s="14">
+        <f>E32+F32</f>
+        <v>37333.333333333336</v>
+      </c>
+      <c r="I32" s="14">
+        <f>E32+F32+G32</f>
+        <v>40333.333333333336</v>
+      </c>
+      <c r="J32" s="14">
+        <f t="shared" si="10"/>
+        <v>62666.666666666664</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10">
       <c r="A33" s="1" t="s">
         <v>19</v>
       </c>
@@ -2873,8 +2983,35 @@
       <c r="C33" s="18">
         <v>45913</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="D33" s="9">
+        <f>J32</f>
+        <v>62666.666666666664</v>
+      </c>
+      <c r="E33" s="7">
+        <f>E32</f>
+        <v>33333.333333333336</v>
+      </c>
+      <c r="F33">
+        <f>F32</f>
+        <v>4000</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33" s="14">
+        <f>H32</f>
+        <v>37333.333333333336</v>
+      </c>
+      <c r="I33" s="14">
+        <f>I32-G32</f>
+        <v>37333.333333333336</v>
+      </c>
+      <c r="J33" s="14">
+        <f t="shared" si="10"/>
+        <v>25333.333333333328</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
       <c r="A34" s="1" t="s">
         <v>19</v>
       </c>
@@ -2884,8 +3021,35 @@
       <c r="C34" s="18">
         <v>45943</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
+      <c r="D34" s="9">
+        <f>J33</f>
+        <v>25333.333333333328</v>
+      </c>
+      <c r="E34" s="7">
+        <f>E33</f>
+        <v>33333.333333333336</v>
+      </c>
+      <c r="F34">
+        <f>F33</f>
+        <v>4000</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34" s="14">
+        <f>H33</f>
+        <v>37333.333333333336</v>
+      </c>
+      <c r="I34" s="14">
+        <f>I33</f>
+        <v>37333.333333333336</v>
+      </c>
+      <c r="J34" s="14">
+        <f t="shared" si="10"/>
+        <v>-12000.000000000007</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
       <c r="A35" s="1" t="s">
         <v>20</v>
       </c>
@@ -2896,7 +3060,7 @@
         <v>45883</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:10">
       <c r="A36" s="1" t="s">
         <v>20</v>
       </c>
@@ -2907,7 +3071,7 @@
         <v>45914</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:10">
       <c r="A37" s="1" t="s">
         <v>64</v>
       </c>
@@ -2918,7 +3082,7 @@
         <v>45944</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:10">
       <c r="A38" s="1" t="s">
         <v>21</v>
       </c>
@@ -2929,7 +3093,7 @@
         <v>45884</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:10">
       <c r="A39" s="1" t="s">
         <v>21</v>
       </c>
@@ -2940,7 +3104,7 @@
         <v>45915</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:10">
       <c r="A40" s="1" t="s">
         <v>21</v>
       </c>
@@ -2951,7 +3115,7 @@
         <v>45945</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:10">
       <c r="A41" s="1" t="s">
         <v>22</v>
       </c>
@@ -2962,7 +3126,7 @@
         <v>45885</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:10">
       <c r="A42" s="1" t="s">
         <v>22</v>
       </c>
@@ -2973,7 +3137,7 @@
         <v>45916</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:10">
       <c r="A43" s="1" t="s">
         <v>22</v>
       </c>
@@ -2984,7 +3148,7 @@
         <v>45946</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:10">
       <c r="A44" s="1" t="s">
         <v>23</v>
       </c>
@@ -2995,7 +3159,7 @@
         <v>45886</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:10">
       <c r="A45" s="1" t="s">
         <v>23</v>
       </c>
@@ -3006,7 +3170,7 @@
         <v>45917</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:10">
       <c r="A46" s="1" t="s">
         <v>23</v>
       </c>
@@ -3017,7 +3181,7 @@
         <v>45947</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:10">
       <c r="A47" s="1" t="s">
         <v>24</v>
       </c>
@@ -3028,7 +3192,7 @@
         <v>45887</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:10">
       <c r="A48" s="1" t="s">
         <v>24</v>
       </c>

</xml_diff>